<commit_message>
Atualiza catÃ¡logo, carrinho e checkout com dados por planilha e correÃ§Ãµes de imagens.
Centraliza a gestÃ£o dos produtos em CSV/JSON, adiciona pÃ¡gina dedicada de carrinho, oculta promo relÃ¢mpago e reforÃ§a fallbacks para caminhos com acentos.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/imagens/docs/Planilha_Produtos.xlsx
+++ b/imagens/docs/Planilha_Produtos.xlsx
@@ -1,26 +1,128 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ikaro\Desktop\caixasecreta\imagens\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646A9DF0-76D2-480A-8ADE-6B673932EEA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{8E8E4DE3-A916-4CC4-810F-212683CE6F7E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>Preço</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Imagem</t>
+  </si>
+  <si>
+    <t>Vibrador Rotativo Vai e Vem com 36 Nível de Pulsação e Estimulador</t>
+  </si>
+  <si>
+    <t>Vibrador Ponto G com Estimulador de Clitóris Língua com 10 Modos de Vibração e Aquecimento</t>
+  </si>
+  <si>
+    <t>Vibradores</t>
+  </si>
+  <si>
+    <t>Vibrador Ponto G com 30 Modos de Vibração</t>
+  </si>
+  <si>
+    <t>Vibrador em Formato de pincel com 8 Modos de Vibração</t>
+  </si>
+  <si>
+    <t>Sophie Vibrador Formato de Rosa com 10 Modos de Vibracao, Vai e Vem e Pulsacao</t>
+  </si>
+  <si>
+    <t>Mini Toy Vibrador Varinha Mágica com 20 Modos de Vibrações e 8 Níveis e Velocidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magesty Vibrador de Calcinha 9 Modos de Pulsação Controle Via APP </t>
+  </si>
+  <si>
+    <t>Estimulador Feminino Porquinho com 10 Modos de Ondas de Pressão</t>
+  </si>
+  <si>
+    <t>Bullet Vibratório com 10 Modos de Vibração Recarregável e Controle por Aplicativo</t>
+  </si>
+  <si>
+    <t>Basebal Bat Vibrador com Aparência Realística com 10 Modos Vai e Vem e Vibração</t>
+  </si>
+  <si>
+    <t>Xana Loka Gel Excitante Feminino Linha Brasileirinhos 15g</t>
+  </si>
+  <si>
+    <t>001 - Vibrador Ponto G em Formato de Golfinho em ABS</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>002</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>Lipstick Vibe Vibrador em Formato de Batom Vibração</t>
+  </si>
+  <si>
+    <t>Preço final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lilo Vibrador Varinha Mágica com 10 Modos de Vibrações </t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -46,13 +148,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -69,7 +175,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -85,7 +191,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -97,7 +203,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -114,7 +220,7 @@
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -144,12 +250,29 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -179,6 +302,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -330,10 +470,224 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8812FC9-AC99-43E8-8307-147C86B4CEF7}">
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="87.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="1">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="1">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="1">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="1">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="1">
+        <v>10.35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="1">
+        <v>79.95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <ignoredErrors>
+    <ignoredError sqref="A2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>